<commit_message>
Add Categories and Expenses modules
- Categories: management page, New Category dialog, Excel read/write
- Expenses: management page with auto VAT total, New Expense dialog with
  mandatory project selection (no save without a project), Excel read/write
- Sidebar: add Categories navigation item
- Tests: safe workbook backup/restore, expense persistence + project requirement
</commit_message>
<xml_diff>
--- a/ONE9SIX9.xlsx
+++ b/ONE9SIX9.xlsx
@@ -455,7 +455,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1"/>
+  <dimension ref="A1:L1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -471,30 +471,50 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
+          <t>Supplier</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Project</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Category</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Invoice/Receipt Number</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
           <t>Description</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>Category</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>Supplier</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>Amount</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Amount Excl. VAT</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>VAT</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>Total Incl. VAT</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
@@ -567,7 +587,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H5"/>
+  <dimension ref="A1:H4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -649,32 +669,15 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>TEST-BUGFIX-001</t>
+          <t>gen</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Bugfix Verification Project</t>
+          <t>general</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
-        <is>
-          <t>Active</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>gen</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>general</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
         <is>
           <t>Completed</t>
         </is>

</xml_diff>

<commit_message>
Dashboard reads live data from Excel
- Expenses This Month sums expenses recorded in the current month
- Net Profit = income minus expenses (income is 0 until built)
- Cards refresh whenever the dashboard is opened
- DashboardCard supports dynamic values; design unchanged
- Tolerant date parsing for free-form dates (e.g. '6 August')
</commit_message>
<xml_diff>
--- a/ONE9SIX9.xlsx
+++ b/ONE9SIX9.xlsx
@@ -455,7 +455,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L1"/>
+  <dimension ref="A1:L2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -518,6 +518,50 @@
         <is>
           <t>Notes</t>
         </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>6 August</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Rio Steel</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>gen — general</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>steel</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>000345</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>steel angle iron and flat bar</t>
+        </is>
+      </c>
+      <c r="H2" t="n">
+        <v>142</v>
+      </c>
+      <c r="I2" t="n">
+        <v>18</v>
+      </c>
+      <c r="J2" t="n">
+        <v>160</v>
       </c>
     </row>
   </sheetData>
@@ -782,7 +826,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D1"/>
+  <dimension ref="A1:D2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -804,6 +848,18 @@
       <c r="D1" t="inlineStr">
         <is>
           <t>Description</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>1969-0005</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>steel</t>
         </is>
       </c>
     </row>

</xml_diff>